<commit_message>
feat: ingest Sep 11 women's-health intel without touching verified deals
Map this week's WH digest onto the catalyst watchlist (Etcamah, LUNA) and a companion brief. Funding, grants, papers, and philanthropy stay intel-only.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1827,37 +1827,37 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>American Regent (Daiichi Sankyo)</t>
+          <t>Alumis</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ALMS</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Injectafer (ferric carboxymaltose) boxed warning</t>
+          <t>envudeucitinib</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>IV iron replacement</t>
+          <t>TYK2 inhibitor</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>iron deficiency anemia</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>systemic lupus erythematosus</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>negative</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>Labeling revision adds boxed warning for severe prolonged symptomatic hypophosphatemia; follows Aug 13 citizen-petition grant; relevant to OB/GYN IV iron use</t>
+          <t>Ph2b LUMUS missed primary and key secondary; high-interferon subgroup active; Ph3 still planned</t>
         </is>
       </c>
     </row>
@@ -1884,37 +1884,37 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Alumis</t>
+          <t>American Regent (Daiichi Sankyo)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ALMS</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>envudeucitinib</t>
+          <t>Injectafer (ferric carboxymaltose) boxed warning</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>TYK2 inhibitor</t>
+          <t>IV iron replacement</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>systemic lupus erythematosus</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>negative</t>
+          <t>iron deficiency anemia</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1924,7 +1924,7 @@
       </c>
       <c r="K25" s="5" t="inlineStr">
         <is>
-          <t>Ph2b LUMUS missed primary and key secondary; high-interferon subgroup active; Ph3 still planned</t>
+          <t>Labeling revision adds boxed warning for severe prolonged symptomatic hypophosphatemia; follows Aug 13 citizen-petition grant; relevant to OB/GYN IV iron use</t>
         </is>
       </c>
     </row>
@@ -2102,47 +2102,47 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Telix</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>TLX</t>
+          <t>AZN</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>TLX101-Px</t>
+          <t>Etcamah (camizestrant)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>PET imaging agent</t>
+          <t>oral SERD</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>glioma imaging</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>ESR1-mutated HR+/HER2- advanced or metastatic breast cancer</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2152,54 +2152,54 @@
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>Radiopharma imaging momentum</t>
+          <t>Accelerated approval Sep 4 2026 with a CDK4/6 inhibitor after ctDNA-detected ESR1 mutation on Guardant360 CDx during AI + CDK4/6 therapy. SERENA-6 (NCT04964934): median PFS 16.0 vs 9.2 months (HR 0.44). First US cancer label triggered by a blood-detected resistance mutation before imaging progression; confirmatory obligation still governs. Not an acquisition.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ABBV</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>CHMP monthly meeting</t>
+          <t>atogepant (QULIPTA/AQUIPTA)</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>oral CGRP receptor antagonist</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>preventive treatment of menstrual migraine</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>Sept 14-17; new opinions resume after August written procedure</t>
+          <t>Phase 3 LUNA topline in 468 patients met the primary endpoint and all eight ranked secondary endpoints. Mean perimenstrual migraine-day reduction 1.20 vs 0.40 placebo. No approved treatment exists for this indication. AbbVie plans worldwide submissions; no PDUFA date yet so this stays a readout row. Sector is Therapeutics: verified taxonomy has no menstrual-health segment.</t>
         </is>
       </c>
     </row>
@@ -2221,37 +2221,37 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
+          <t>Telix</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TLX</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Pediatric Advisory Committee</t>
+          <t>TLX101-Px</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>PET imaging agent</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>glioma imaging</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Virtual session</t>
+          <t>Radiopharma imaging momentum</t>
         </is>
       </c>
     </row>
@@ -2278,37 +2278,37 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Ultragenyx/Abeona</t>
+          <t>EMA</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>RARE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>UX111</t>
+          <t>CHMP monthly meeting</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>AAV gene therapy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Sanfilippo syndrome type A</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Second RARE gene-therapy decision in ~1 month</t>
+          <t>Sept 14-17; new opinions resume after August written procedure</t>
         </is>
       </c>
     </row>
@@ -2335,37 +2335,37 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Merck</t>
+          <t>FDA</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Winrevair (sotatercept) sNDA</t>
+          <t>Pediatric Advisory Committee</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>activin signaling inhibitor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>PAH earlier-line (HYPERION)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Label expansion</t>
+          <t>Virtual session</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2402,32 +2402,32 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ionis</t>
+          <t>Ultragenyx/Abeona</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>IONS</t>
+          <t>RARE</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>zilganersen</t>
+          <t>UX111</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>AAV gene therapy</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Alexander disease</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>Sanfilippo syndrome type A</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2437,7 +2437,7 @@
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
+          <t>Second RARE gene-therapy decision in ~1 month</t>
         </is>
       </c>
     </row>
@@ -2449,37 +2449,37 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
+          <t>Merck</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Galleri MCED test</t>
+          <t>Winrevair (sotatercept) sNDA</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>multi-cancer early detection</t>
+          <t>activin signaling inhibitor</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>cancer screening</t>
+          <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+          <t>Label expansion</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2516,32 +2516,32 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Incyte/Mirum</t>
+          <t>Ionis</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>IONS</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>zilganersen</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>ALK2 inhibitor</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>anemia of myelofibrosis</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>Alexander disease</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -2551,49 +2551,49 @@
       </c>
       <c r="K36" s="5" t="inlineStr">
         <is>
-          <t>Per pdufa.bio calendar</t>
+          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>Galleri MCED test</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>multi-cancer early detection</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>actinic keratosis</t>
+          <t>cancer screening</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2608,19 +2608,19 @@
       </c>
       <c r="K37" s="5" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2630,27 +2630,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Incyte/Mirum</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>INCY</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>ALK2 inhibitor</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
+          <t>anemia of myelofibrosis</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2665,19 +2665,19 @@
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>Per pdufa.bio calendar</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2687,32 +2687,32 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>actinic keratosis</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -2722,14 +2722,14 @@
       </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>Device-drug combination label expansion</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2744,27 +2744,27 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
+          <t>hemophilia A</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr">
         <is>
-          <t>US decision after EU MAA withdrawal in Aug 2026</t>
+          <t>Next-gen challenger to Hemlibra</t>
         </is>
       </c>
     </row>
@@ -2843,12 +2843,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2858,32 +2858,32 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>polycythemia vera</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -2893,19 +2893,19 @@
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2915,27 +2915,27 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
+          <t>spinal muscular atrophy</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -2950,19 +2950,19 @@
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>US decision after EU MAA withdrawal in Aug 2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2982,17 +2982,17 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>IL-6 receptor antagonist</t>
+          <t>PD-L1 checkpoint inhibitor</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
+          <t>stage III colon cancer</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
@@ -3007,19 +3007,19 @@
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>Checkpoint expansion into adjuvant colon</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3029,27 +3029,27 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Merck/Daiichi Sankyo</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>B7-H3 antibody-drug conjugate</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
+          <t>extensive-stage small cell lung cancer</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>Label expansion for Joenja</t>
+          <t>First regulatory decision for a B7-H3 ADC</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3086,27 +3086,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>Enspryng (satralizumab)</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>IL-6 receptor antagonist</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
+          <t>thyroid eye disease</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -3121,62 +3121,176 @@
       </c>
       <c r="K46" s="5" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>First IL-6R challenger to Tepezza</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Pharming</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>PHAR</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>leniolisib</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>PI3K-delta inhibitor</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Label expansion for Joenja</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>bepirovirsen</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>antisense oligonucleotide</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>chronic hepatitis B</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>B-Well program; functional-cure ambition in HBV</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Capricor</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>CAPR</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>deramiocel</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>allogeneic cell therapy</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>DMD cardiomyopathy</t>
         </is>
       </c>
-      <c r="I47" s="8" t="inlineStr">
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>delayed</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K47" s="5" t="inlineStr">
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
         <is>
           <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
@@ -3231,6 +3345,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: weekly biopharma brief 2026-09-18 and watchlist update
- Resolve 5 events: Pixclara approved 9/11 (announced 9/14), FAYUVI (UX111)
  approved 9/17 two days early, zipalertinib REZILIENT3 positive, CHMP Sept
  plenary, Pediatric AdComm.
- Correct zilurgisertib indication: fibrodysplasia ossificans progressiva, not
  anemia of myelofibrosis (third aggregator-sourced error in this file).
- Add 8 rows incl. three women's-health CHMP opinions (relacorilant, senaparib,
  pertuzumab biosimilar) and the MIUDELLA 6-year sNDA.
- 54 -> 62 rows; women's-health-relevant 2 -> 6. Regenerate catalysts.xlsx.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>TLX101-Px</t>
+          <t>TLX101-Px (Pixclara, floretyrosine F 18)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -2334,9 +2334,9 @@
           <t>glioma imaging</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>PDUFA date of Sep 11 2026 passed with no approval or CRL announced as of that evening; row deliberately left upcoming rather than inferred. Telix previously received a CRL on the related glioma imaging NDA TLX101-CDx, so silence is not directional</t>
+          <t>Approved; FDA novel-approval list dates it 9/11/2026 (entry #40) while Telix announced Sep 14 - a 3-day disclosure lag, which is why last week's brief correctly left the row unresolved. First FDA-approved FET-PET imaging drug for glioma; adults and pediatric patients 1 month and older.</t>
         </is>
       </c>
     </row>
@@ -2391,9 +2391,9 @@
           <t>first-line EGFR exon 20 insertion mutation NSCLC</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 REZILIENT3 planned interim analysis of zipalertinib plus chemotherapy, Presidential Symposium 2 at IASLC WCLC 2026 in Seoul</t>
+          <t>REZILIENT3 (NCT05973773) interim met primary endpoint: mPFS 14.5 mo (95% CI 12.9-21.4) vs 8.5 mo (7.0-10.9), HR 0.50 (0.34-0.73), p=0.00015, BICR, data cut 29 May 2026. Tolerability is the offset: grade &gt;=3 treatment-related AEs 80.7% vs 40.4% and 3 treatment-related deaths (2.1%) vs none.</t>
         </is>
       </c>
     </row>
@@ -2448,9 +2448,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
@@ -2460,54 +2460,54 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Sept 14-17; new opinions resume after August written procedure</t>
+          <t>Sept 14-17 plenary: 12 new medicines recommended (incl. Frehemgo/denecimig, Lifyorli/relacorilant, Sepalna/senaparib, Pebrilzo pertuzumab biosimilar) plus 10 extensions of indication; zero negative opinions on new medicines (8 YTD); Xervyteg refusal confirmed on re-examination; Isembyld (apitegromab) and Zinmyleo initial applications withdrawn; Alhemo, Kaftrio and Kalydeco pediatric extensions withdrawn.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
+          <t>Vera Therapeutics</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VERA</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Pediatric Advisory Committee</t>
+          <t>atacicept-vymj (TRUTAKNA)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dual BLyS/APRIL inhibitor fusion protein</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Virtual session</t>
+          <t>ORIGIN 3 final 104-week efficacy analysis. Composite kidney-disease progression: 11 vs 38 events, HR 0.24 (95% CI 0.12-0.48), 76% risk reduction, p&lt;0.0001. Annualized eGFR slope -0.6 (95% CI -1.6, 0.4) vs -5.6 (-6.6, -4.6) mL/min/1.73m2/yr, treatment effect 5.0. Dialysis &gt;=30 days, transplant or death: 0 vs 8. Converts the July 2026 accelerated approval into a full-approval filing; sBLA planned Q4 2026.</t>
         </is>
       </c>
     </row>
@@ -2529,42 +2529,42 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Ultragenyx/Abeona</t>
+          <t>FDA</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>RARE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>UX111</t>
+          <t>Pediatric Advisory Committee</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>AAV gene therapy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Sanfilippo syndrome type A</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -2574,54 +2574,50 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Second RARE gene-therapy decision in ~1 month</t>
+          <t>Held. FDA's postmarketing pediatric safety reviews identified no new safety signals in 14 of the products reviewed (Sprycel handled separately). No label actions recommended out of the session.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Merck</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
+          <t>Biosimilar Collaborations Ireland</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Winrevair (sotatercept-csrk) sBLA</t>
+          <t>pertuzumab biosimilar (Pebrilzo)</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>activin signaling inhibitor</t>
+          <t>anti-HER2 monoclonal antibody biosimilar</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>PAH earlier-line (HYPERION)</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>HER2-positive early and metastatic breast cancer</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -2631,54 +2627,54 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
+          <t>EMA states Pebrilzo is the first biosimilar recommended for approval following the tailored clinical approach - the reflection paper finalised 16 Mar 2026 under which comparative efficacy studies may be waived for well-characterised substances when analytical comparability plus PK and safety data are more sensitive. Precedent for biosimilar development cost, not for pertuzumab specifically: Henlius/Organon POHERDY was already the first EU pertuzumab biosimilar (EC approval 29 Apr 2026).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Ionis</t>
+          <t>Corcept Therapeutics</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>IONS</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>zilganersen</t>
+          <t>relacorilant (Lifyorli)</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>selective glucocorticoid receptor modulator</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Alexander disease</t>
+          <t>platinum-resistant high-grade epithelial ovarian, fallopian tube or primary peritoneal cancer, with nab-paclitaxel</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
@@ -2688,54 +2684,50 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
+          <t>Positive CHMP opinion for patients who have had one to three prior systemic regimens; EC decision pending. Cortisol-modulation mechanism is orthogonal to PARP and anti-angiogenics, so it widens rather than crowds the platinum-resistant option set.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>GRAL</t>
-        </is>
-      </c>
+          <t>SFL Pharmaceuticals Deutschland</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Galleri MCED test</t>
+          <t>senaparib (Sepalna)</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>multi-cancer early detection</t>
+          <t>PARP inhibitor</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>cancer screening</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>maintenance treatment of advanced high-grade epithelial ovarian, fallopian tube or primary peritoneal cancer</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -2745,7 +2737,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+          <t>Positive CHMP opinion; EC decision pending. Applicant of record is SFL Pharmaceuticals Deutschland GmbH per EMA. Adds a further PARP inhibitor to EU ovarian maintenance, where pricing pressure already outweighs mechanism novelty.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2749,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2767,32 +2759,32 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Incyte/Mirum</t>
+          <t>Ultragenyx/Abeona</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>RARE</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>UX111 (FAYUVI, rebisufligene etisparvovec-hopf)</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>ALK2 inhibitor</t>
+          <t>AAV gene therapy</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>anemia of myelofibrosis</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>Sanfilippo syndrome type A</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
@@ -2802,19 +2794,19 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Per pdufa.bio calendar</t>
+          <t>Approved Sep 17, two days ahead of the Sep 19 goal date. First-ever FDA-approved treatment for Sanfilippo syndrome Type A (MPS IIIA), for neurologic manifestations in pediatric patients with preserved neurodevelopmental function. Follows a prior CRL; priority review voucher granted. EU path diverges - see CHMP Sep 2026.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2824,27 +2816,27 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Merck</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>Winrevair (sotatercept-csrk) sBLA</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>activin signaling inhibitor</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>actinic keratosis</t>
+          <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2859,19 +2851,19 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion</t>
+          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2881,32 +2873,32 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Ionis</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>IONS</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>zilganersen</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>Alexander disease</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
@@ -2916,7 +2908,7 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
         </is>
       </c>
     </row>
@@ -2928,42 +2920,42 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Galleri MCED test</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>multi-cancer early detection</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>cancer screening</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2973,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2977,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2995,32 +2987,32 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3030,19 +3022,19 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3052,32 +3044,32 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>actinic keratosis</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -3087,14 +3079,14 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Device-drug combination label expansion</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3104,32 +3096,32 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>hemophilia A</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -3144,50 +3136,54 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
+          <t>Next-gen challenger to Hemlibra</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>Priovant/Roivant</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>dermatomyositis</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3197,19 +3193,19 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3219,32 +3215,32 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
-        </is>
-      </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>polycythemia vera</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3254,19 +3250,19 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3276,32 +3272,32 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>spinal muscular atrophy</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
@@ -3311,49 +3307,49 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>IL-6 receptor antagonist</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
+          <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -3368,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
         </is>
       </c>
     </row>
@@ -3380,37 +3376,33 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>VTRS</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3425,19 +3417,19 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3447,32 +3439,32 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>PD-L1 checkpoint inhibitor</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3482,19 +3474,19 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>Checkpoint expansion into adjuvant colon</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3504,27 +3496,27 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Merck/Daiichi Sankyo</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>B7-H3 antibody-drug conjugate</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
+          <t>extensive-stage small cell lung cancer</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3539,49 +3531,41 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>First regulatory decision for a B7-H3 ADC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>INO</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr">
@@ -3596,69 +3580,517 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Enspryng (satralizumab)</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>IL-6 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>First IL-6R challenger to Tepezza</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Viatris/Opus Genetics</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>alpha-adrenergic antagonist eye drop</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>presbyopia</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Pharming</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>PHAR</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>leniolisib</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>PI3K-delta inhibitor</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>bepirovirsen</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>antisense oligonucleotide</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>chronic hepatitis B</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>B-Well program; functional-cure ambition in HBV</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Inovio</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>INO-3107</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>recurrent respiratory papillomatosis</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Vaxcyte</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>VAX-31</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>31-valent pneumococcal conjugate vaccine</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>adult pneumococcal disease prevention</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>AdComm</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Capricor</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>CAPR</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>deramiocel</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>allogeneic cell therapy</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>DMD cardiomyopathy</t>
         </is>
       </c>
-      <c r="I55" s="9" t="inlineStr">
+      <c r="I62" s="9" t="inlineStr">
         <is>
           <t>delayed</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
         <is>
           <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Organon/Sebela Women's Health</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>MIUDELLA (copper intrauterine system)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>hormone-free copper intrauterine device</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>prevention of pregnancy - extension of duration of use to 6 years</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K55"/>
+  <autoFilter ref="A1:K63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -3714,6 +4146,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: weekly biopharma brief 2026-09-18 and watchlist update (#208)
- Resolve 5 events: Pixclara approved 9/11 (announced 9/14), FAYUVI (UX111)
  approved 9/17 two days early, zipalertinib REZILIENT3 positive, CHMP Sept
  plenary, Pediatric AdComm.
- Correct zilurgisertib indication: fibrodysplasia ossificans progressiva, not
  anemia of myelofibrosis (third aggregator-sourced error in this file).
- Add 8 rows incl. three women's-health CHMP opinions (relacorilant, senaparib,
  pertuzumab biosimilar) and the MIUDELLA 6-year sNDA.
- 54 -> 62 rows; women's-health-relevant 2 -> 6. Regenerate catalysts.xlsx.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2321,7 +2321,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>TLX101-Px</t>
+          <t>TLX101-Px (Pixclara, floretyrosine F 18)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -2334,9 +2334,9 @@
           <t>glioma imaging</t>
         </is>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>PDUFA date of Sep 11 2026 passed with no approval or CRL announced as of that evening; row deliberately left upcoming rather than inferred. Telix previously received a CRL on the related glioma imaging NDA TLX101-CDx, so silence is not directional</t>
+          <t>Approved; FDA novel-approval list dates it 9/11/2026 (entry #40) while Telix announced Sep 14 - a 3-day disclosure lag, which is why last week's brief correctly left the row unresolved. First FDA-approved FET-PET imaging drug for glioma; adults and pediatric patients 1 month and older.</t>
         </is>
       </c>
     </row>
@@ -2391,9 +2391,9 @@
           <t>first-line EGFR exon 20 insertion mutation NSCLC</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 REZILIENT3 planned interim analysis of zipalertinib plus chemotherapy, Presidential Symposium 2 at IASLC WCLC 2026 in Seoul</t>
+          <t>REZILIENT3 (NCT05973773) interim met primary endpoint: mPFS 14.5 mo (95% CI 12.9-21.4) vs 8.5 mo (7.0-10.9), HR 0.50 (0.34-0.73), p=0.00015, BICR, data cut 29 May 2026. Tolerability is the offset: grade &gt;=3 treatment-related AEs 80.7% vs 40.4% and 3 treatment-related deaths (2.1%) vs none.</t>
         </is>
       </c>
     </row>
@@ -2448,9 +2448,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
@@ -2460,54 +2460,54 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Sept 14-17; new opinions resume after August written procedure</t>
+          <t>Sept 14-17 plenary: 12 new medicines recommended (incl. Frehemgo/denecimig, Lifyorli/relacorilant, Sepalna/senaparib, Pebrilzo pertuzumab biosimilar) plus 10 extensions of indication; zero negative opinions on new medicines (8 YTD); Xervyteg refusal confirmed on re-examination; Isembyld (apitegromab) and Zinmyleo initial applications withdrawn; Alhemo, Kaftrio and Kalydeco pediatric extensions withdrawn.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
+          <t>Vera Therapeutics</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VERA</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Pediatric Advisory Committee</t>
+          <t>atacicept-vymj (TRUTAKNA)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dual BLyS/APRIL inhibitor fusion protein</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Virtual session</t>
+          <t>ORIGIN 3 final 104-week efficacy analysis. Composite kidney-disease progression: 11 vs 38 events, HR 0.24 (95% CI 0.12-0.48), 76% risk reduction, p&lt;0.0001. Annualized eGFR slope -0.6 (95% CI -1.6, 0.4) vs -5.6 (-6.6, -4.6) mL/min/1.73m2/yr, treatment effect 5.0. Dialysis &gt;=30 days, transplant or death: 0 vs 8. Converts the July 2026 accelerated approval into a full-approval filing; sBLA planned Q4 2026.</t>
         </is>
       </c>
     </row>
@@ -2529,42 +2529,42 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Ultragenyx/Abeona</t>
+          <t>FDA</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>RARE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>UX111</t>
+          <t>Pediatric Advisory Committee</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>AAV gene therapy</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Sanfilippo syndrome type A</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -2574,54 +2574,50 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Second RARE gene-therapy decision in ~1 month</t>
+          <t>Held. FDA's postmarketing pediatric safety reviews identified no new safety signals in 14 of the products reviewed (Sprycel handled separately). No label actions recommended out of the session.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Merck</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>MRK</t>
-        </is>
-      </c>
+          <t>Biosimilar Collaborations Ireland</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Winrevair (sotatercept-csrk) sBLA</t>
+          <t>pertuzumab biosimilar (Pebrilzo)</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>activin signaling inhibitor</t>
+          <t>anti-HER2 monoclonal antibody biosimilar</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>PAH earlier-line (HYPERION)</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>HER2-positive early and metastatic breast cancer</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -2631,54 +2627,54 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
+          <t>EMA states Pebrilzo is the first biosimilar recommended for approval following the tailored clinical approach - the reflection paper finalised 16 Mar 2026 under which comparative efficacy studies may be waived for well-characterised substances when analytical comparability plus PK and safety data are more sensitive. Precedent for biosimilar development cost, not for pertuzumab specifically: Henlius/Organon POHERDY was already the first EU pertuzumab biosimilar (EC approval 29 Apr 2026).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Ionis</t>
+          <t>Corcept Therapeutics</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>IONS</t>
+          <t>CORT</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>zilganersen</t>
+          <t>relacorilant (Lifyorli)</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>selective glucocorticoid receptor modulator</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>Alexander disease</t>
+          <t>platinum-resistant high-grade epithelial ovarian, fallopian tube or primary peritoneal cancer, with nab-paclitaxel</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
@@ -2688,54 +2684,50 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
+          <t>Positive CHMP opinion for patients who have had one to three prior systemic regimens; EC decision pending. Cortisol-modulation mechanism is orthogonal to PARP and anti-angiogenics, so it widens rather than crowds the platinum-resistant option set.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>GRAL</t>
-        </is>
-      </c>
+          <t>SFL Pharmaceuticals Deutschland</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr"/>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Galleri MCED test</t>
+          <t>senaparib (Sepalna)</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>multi-cancer early detection</t>
+          <t>PARP inhibitor</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>cancer screening</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>maintenance treatment of advanced high-grade epithelial ovarian, fallopian tube or primary peritoneal cancer</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
@@ -2745,7 +2737,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+          <t>Positive CHMP opinion; EC decision pending. Applicant of record is SFL Pharmaceuticals Deutschland GmbH per EMA. Adds a further PARP inhibitor to EU ovarian maintenance, where pricing pressure already outweighs mechanism novelty.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2749,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2767,32 +2759,32 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Incyte/Mirum</t>
+          <t>Ultragenyx/Abeona</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>RARE</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>UX111 (FAYUVI, rebisufligene etisparvovec-hopf)</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>ALK2 inhibitor</t>
+          <t>AAV gene therapy</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>anemia of myelofibrosis</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>Sanfilippo syndrome type A</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
@@ -2802,19 +2794,19 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Per pdufa.bio calendar</t>
+          <t>Approved Sep 17, two days ahead of the Sep 19 goal date. First-ever FDA-approved treatment for Sanfilippo syndrome Type A (MPS IIIA), for neurologic manifestations in pediatric patients with preserved neurodevelopmental function. Follows a prior CRL; priority review voucher granted. EU path diverges - see CHMP Sep 2026.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2824,27 +2816,27 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Merck</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>Winrevair (sotatercept-csrk) sBLA</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>activin signaling inhibitor</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>actinic keratosis</t>
+          <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2859,19 +2851,19 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion</t>
+          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2881,32 +2873,32 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Ionis</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>IONS</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>zilganersen</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>Alexander disease</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
@@ -2916,7 +2908,7 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
         </is>
       </c>
     </row>
@@ -2928,42 +2920,42 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Galleri MCED test</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>multi-cancer early detection</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>cancer screening</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2973,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2977,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2995,32 +2987,32 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3030,19 +3022,19 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3052,32 +3044,32 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>actinic keratosis</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -3087,14 +3079,14 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Device-drug combination label expansion</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3104,32 +3096,32 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>hemophilia A</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -3144,50 +3136,54 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
+          <t>Next-gen challenger to Hemlibra</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>Priovant/Roivant</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>ROIV</t>
+        </is>
+      </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>dermatomyositis</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3197,19 +3193,19 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3219,32 +3215,32 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
-        </is>
-      </c>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>polycythemia vera</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3254,19 +3250,19 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3276,32 +3272,32 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>spinal muscular atrophy</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J49" s="5" t="inlineStr">
@@ -3311,49 +3307,49 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>IL-6 receptor antagonist</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
+          <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -3368,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
         </is>
       </c>
     </row>
@@ -3380,37 +3376,33 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>VTRS</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr"/>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3425,19 +3417,19 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -3447,32 +3439,32 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>PD-L1 checkpoint inhibitor</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3482,19 +3474,19 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>Checkpoint expansion into adjuvant colon</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -3504,27 +3496,27 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Merck/Daiichi Sankyo</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>B7-H3 antibody-drug conjugate</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
+          <t>extensive-stage small cell lung cancer</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3539,49 +3531,41 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>First regulatory decision for a B7-H3 ADC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>INO</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr"/>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr">
@@ -3596,69 +3580,517 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Enspryng (satralizumab)</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>IL-6 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>First IL-6R challenger to Tepezza</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Viatris/Opus Genetics</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>alpha-adrenergic antagonist eye drop</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>presbyopia</t>
+        </is>
+      </c>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Pharming</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>PHAR</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>leniolisib</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>PI3K-delta inhibitor</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>bepirovirsen</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>antisense oligonucleotide</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>chronic hepatitis B</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>B-Well program; functional-cure ambition in HBV</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Inovio</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>INO-3107</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>recurrent respiratory papillomatosis</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Vaxcyte</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>VAX-31</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>31-valent pneumococcal conjugate vaccine</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>adult pneumococcal disease prevention</t>
+        </is>
+      </c>
+      <c r="I60" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>AdComm</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr"/>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+        </is>
+      </c>
+      <c r="I61" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Capricor</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>CAPR</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F62" s="3" t="inlineStr">
         <is>
           <t>deramiocel</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>allogeneic cell therapy</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>DMD cardiomyopathy</t>
         </is>
       </c>
-      <c r="I55" s="9" t="inlineStr">
+      <c r="I62" s="9" t="inlineStr">
         <is>
           <t>delayed</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr">
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
         <is>
           <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Organon/Sebela Women's Health</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>OGN</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>MIUDELLA (copper intrauterine system)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>hormone-free copper intrauterine device</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>prevention of pregnancy - extension of duration of use to 6 years</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K55"/>
+  <autoFilter ref="A1:K63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -3714,6 +4146,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: catch-up weekly brief + watchlist (Sep 19–Oct 13 2026)
Resolves 9 overdue catalysts (Winrevair, Galleri AdComm, zilurgisertib,
Ameluz, Mim8 delay, inaxaplin, VRBPAC, Tecentriq, I-DXd withdrawal), adds 12
upcoming rows (62 -> 74), regenerates catalysts.xlsx, adds briefs/2026-10-13.md.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2839,9 +2839,9 @@
           <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
+          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363 | Approved Sep 21 2026 (sBLA S-012 letter); label adds HYPERION data, HR 0.24 for clinical worsening in newly diagnosed PAH.</t>
         </is>
       </c>
     </row>
@@ -2953,9 +2953,9 @@
           <t>cancer screening</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
         </is>
       </c>
     </row>
@@ -3010,9 +3010,9 @@
           <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
@@ -3064,12 +3064,12 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>actinic keratosis</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
@@ -3124,9 +3124,9 @@
           <t>hemophilia A</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3352,9 +3352,9 @@
           <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | Resolved by Phase 2b AMPLIFIED (not AMPLITUDE): UACR -42.7% modest-proteinuria cohort, -17.3% T2D cohort (CI crosses 0). AMPLITUDE interim analysis tracked as separate row.</t>
         </is>
       </c>
     </row>
@@ -3405,9 +3405,9 @@
           <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
@@ -3462,9 +3462,9 @@
           <t>stage III colon cancer</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
@@ -3519,9 +3519,9 @@
           <t>extensive-stage small cell lung cancer</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions.</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3768,32 +3768,28 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>GSK</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3808,19 +3804,19 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3830,27 +3826,27 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3865,49 +3861,49 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>Inovio</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>INO-3107</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3922,7 +3918,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
         </is>
       </c>
     </row>
@@ -3934,29 +3930,37 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr"/>
+          <t>Vaxcyte</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr"/>
+          <t>VAX-31</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>31-valent pneumococcal conjugate vaccine</t>
+        </is>
+      </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>adult pneumococcal disease prevention</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3971,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3993,32 +3997,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>CAPR</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>sickle cell disease (RISE UP)</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -4026,71 +4030,727 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
-        </is>
-      </c>
+      <c r="K62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Cytokinetics</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>CYTK</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>aficamten (MAPLE-HCM)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>cardiac myosin inhibitor</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>SMMT</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>ivonescimab</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>PD-1 x VEGF bispecific antibody</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>AdComm</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Capricor</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>deramiocel</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>allogeneic cell therapy</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Savara</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>SVRA</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>MOLBREEVI (molgramostim)</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>inhaled GM-CSF</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>BridgeBio</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>BBIO</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>BBP-418 (ribitol)</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>glycosylation substrate</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Cogent</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>COGT</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>bezuclastinib + sunitinib</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>KIT inhibitor</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant (adjuvant)</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>povetacicept (ALPN-303)</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>dual BAFF/APRIL inhibitor</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant + everolimus</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD + mTOR inhibitor</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F75" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G75" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I63" s="6" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J63" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K63"/>
+  <autoFilter ref="A1:K75"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -4154,6 +4814,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: catch-up weekly brief + watchlist (Sep 19–Oct 13 2026) (#281)
Resolves 9 overdue catalysts (Winrevair, Galleri AdComm, zilurgisertib,
Ameluz, Mim8 delay, inaxaplin, VRBPAC, Tecentriq, I-DXd withdrawal), adds 12
upcoming rows (62 -> 74), regenerates catalysts.xlsx, adds briefs/2026-10-13.md.

Co-authored-by: maekass <234696301+maekass@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2839,9 +2839,9 @@
           <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
+          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363 | Approved Sep 21 2026 (sBLA S-012 letter); label adds HYPERION data, HR 0.24 for clinical worsening in newly diagnosed PAH.</t>
         </is>
       </c>
     </row>
@@ -2953,9 +2953,9 @@
           <t>cancer screening</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
         </is>
       </c>
     </row>
@@ -3010,9 +3010,9 @@
           <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
@@ -3064,12 +3064,12 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>actinic keratosis</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
@@ -3124,9 +3124,9 @@
           <t>hemophilia A</t>
         </is>
       </c>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3352,9 +3352,9 @@
           <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | Resolved by Phase 2b AMPLIFIED (not AMPLITUDE): UACR -42.7% modest-proteinuria cohort, -17.3% T2D cohort (CI crosses 0). AMPLITUDE interim analysis tracked as separate row.</t>
         </is>
       </c>
     </row>
@@ -3405,9 +3405,9 @@
           <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
@@ -3462,9 +3462,9 @@
           <t>stage III colon cancer</t>
         </is>
       </c>
-      <c r="I52" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
@@ -3519,9 +3519,9 @@
           <t>extensive-stage small cell lung cancer</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions.</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3768,32 +3768,28 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>GSK</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3808,19 +3804,19 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3830,27 +3826,27 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3865,49 +3861,49 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>Inovio</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>INO-3107</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3922,7 +3918,7 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
         </is>
       </c>
     </row>
@@ -3934,29 +3930,37 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr"/>
+          <t>Vaxcyte</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>PCVX</t>
+        </is>
+      </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr"/>
+          <t>VAX-31</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>31-valent pneumococcal conjugate vaccine</t>
+        </is>
+      </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>adult pneumococcal disease prevention</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3971,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3993,32 +3997,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>CAPR</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I62" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>sickle cell disease (RISE UP)</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -4026,71 +4030,727 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr">
-        <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
-        </is>
-      </c>
+      <c r="K62" s="3" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Cytokinetics</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>CYTK</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>aficamten (MAPLE-HCM)</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>cardiac myosin inhibitor</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-14</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Summit</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>SMMT</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>ivonescimab</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>PD-1 x VEGF bispecific antibody</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
+        </is>
+      </c>
+      <c r="I64" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>AdComm</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Capricor</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>CAPR</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>deramiocel</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>allogeneic cell therapy</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Savara</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>SVRA</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>MOLBREEVI (molgramostim)</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>inhaled GM-CSF</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
+        </is>
+      </c>
+      <c r="I67" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>BridgeBio</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>BBIO</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>BBP-418 (ribitol)</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>glycosylation substrate</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Cogent</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>COGT</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>bezuclastinib + sunitinib</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>KIT inhibitor</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
+        </is>
+      </c>
+      <c r="I69" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant (adjuvant)</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>povetacicept (ALPN-303)</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>dual BAFF/APRIL inhibitor</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant + everolimus</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD + mTOR inhibitor</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F75" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G63" s="3" t="inlineStr">
+      <c r="G75" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I63" s="6" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J63" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K63"/>
+  <autoFilter ref="A1:K75"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -4154,6 +4814,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: split inaxaplin Phase 2b/Phase 3 catalysts and add Tukysa approval row
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2915,42 +2915,42 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Galleri MCED test</t>
+          <t>inaxaplin (AMPLIFIED Phase 2b)</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>multi-cancer early detection</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>cancer screening</t>
+          <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
+          <t>Phase 2b AMPLIFIED topline: UACR -42.7% in the modest-proteinuria cohort, -17.3% in the T2D cohort (CI crosses 0). Not the Phase 3 AMPLITUDE readout - see the 2026-09-30 and 2027-01-01 rows.</t>
         </is>
       </c>
     </row>
@@ -2977,42 +2977,42 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Mirum/Incyte</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>MIRM</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>Galleri MCED test</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>oral ALK2 kinase inhibitor</t>
+          <t>multi-cancer early detection</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+          <t>cancer screening</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3022,19 +3022,19 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3044,27 +3044,27 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>superficial basal cell carcinoma (sBCC)</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3079,19 +3079,19 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3101,32 +3101,32 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I46" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3136,14 +3136,14 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3158,32 +3158,32 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>hemophilia A</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3215,27 +3215,27 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Priovant/Roivant</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
+          <t>dermatomyositis</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
@@ -3272,27 +3272,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
+          <t>polycythemia vera</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3307,14 +3307,14 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3324,37 +3324,37 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>spinal muscular atrophy</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | Resolved by Phase 2b AMPLIFIED (not AMPLITUDE): UACR -42.7% modest-proteinuria cohort, -17.3% T2D cohort (CI crosses 0). AMPLITUDE interim analysis tracked as separate row.</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
@@ -3376,38 +3376,42 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>positive</t>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3417,54 +3421,50 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,54 +3474,54 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>Tukysa (tucatinib)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>HER2-selective tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I53" s="7" t="inlineStr">
-        <is>
-          <t>withdrawn</t>
+          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,46 +3531,54 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
+          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>CHMP monthly meeting</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr"/>
+          <t>Tecentriq (atezolizumab)</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>PD-L1 checkpoint inhibitor</t>
+        </is>
+      </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
@@ -3580,19 +3588,19 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3602,32 +3610,32 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Merck/Daiichi Sankyo</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>IL-6 receptor antagonist</t>
+          <t>B7-H3 antibody-drug conjugate</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>extensive-stage small cell lung cancer</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3637,49 +3645,41 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>VTRS</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3716,32 +3716,32 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Enspryng (satralizumab)</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>IL-6 receptor antagonist</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3751,45 +3751,49 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>First IL-6R challenger to Tepezza</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>guidance</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr"/>
+          <t>Viatris/Opus Genetics</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>BsUFA IV reauthorization public meeting</t>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>biosimilars</t>
+          <t>alpha-adrenergic antagonist eye drop</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>presbyopia</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3804,7 +3808,7 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3820,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3826,32 +3830,32 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Pharming</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>PHAR</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>leniolisib</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>PI3K-delta inhibitor</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
-        </is>
-      </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3861,49 +3865,45 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>INO</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3918,49 +3918,49 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3975,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3997,27 +3997,27 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Agios</t>
+          <t>Inovio</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>mitapivat (PYRUKYND)</t>
+          <t>INO-3107</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>pyruvate kinase activator</t>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>sickle cell disease (RISE UP)</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -4030,47 +4030,51 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr"/>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Cytokinetics</t>
+          <t>Vaxcyte</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>CYTK</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>aficamten (MAPLE-HCM)</t>
+          <t>VAX-31</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>cardiac myosin inhibitor</t>
+          <t>31-valent pneumococcal conjugate vaccine</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>obstructive HCM (MAPLE-HCM label update)</t>
+          <t>adult pneumococcal disease prevention</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -4083,7 +4087,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4093,7 +4101,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4103,27 +4111,27 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Summit</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>ivonescimab</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>PD-1 x VEGF bispecific antibody</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>EGFR-mutant NSCLC with platinum doublet</t>
+          <t>sickle cell disease (RISE UP)</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -4136,43 +4144,47 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t>First US filing for the PD-1/VEGF bispecific class.</t>
-        </is>
-      </c>
+      <c r="K64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>Cytokinetics</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>CYTK</t>
+        </is>
+      </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr"/>
+          <t>aficamten (MAPLE-HCM)</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>cardiac myosin inhibitor</t>
+        </is>
+      </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -4185,21 +4197,17 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
-        </is>
-      </c>
+      <c r="K65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4209,32 +4217,32 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
+          <t>Summit</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>CAPR</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>ivonescimab</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>PD-1 x VEGF bispecific antibody</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I66" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -4244,49 +4252,41 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Savara</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>SVRA</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>MOLBREEVI (molgramostim)</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>inhaled GM-CSF</t>
-        </is>
-      </c>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>autoimmune pulmonary alveolar proteinosis</t>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4301,19 +4301,19 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -4323,32 +4323,32 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>BridgeBio</t>
+          <t>Capricor</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>CAPR</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>BBP-418 (ribitol)</t>
+          <t>deramiocel</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>glycosylation substrate</t>
+          <t>allogeneic cell therapy</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
-        </is>
-      </c>
-      <c r="I68" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4356,7 +4356,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4366,7 +4370,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -4376,27 +4380,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Cogent</t>
+          <t>Savara</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>bezuclastinib + sunitinib</t>
+          <t>MOLBREEVI (molgramostim)</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>KIT inhibitor</t>
+          <t>inhaled GM-CSF</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>gastrointestinal stromal tumor (PEAK)</t>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -4411,7 +4415,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4427,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4433,27 +4437,27 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>BridgeBio</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>giredestrant (adjuvant)</t>
+          <t>BBP-418 (ribitol)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>oral SERD</t>
+          <t>glycosylation substrate</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4466,11 +4470,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
-        </is>
-      </c>
+      <c r="K70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4490,27 +4490,27 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Cogent</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>povetacicept (ALPN-303)</t>
+          <t>bezuclastinib + sunitinib</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>dual BAFF/APRIL inhibitor</t>
+          <t>KIT inhibitor</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>IgA nephropathy</t>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4523,7 +4523,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4533,7 +4537,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4553,17 +4557,17 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>giredestrant + everolimus</t>
+          <t>giredestrant (adjuvant)</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>oral SERD + mTOR inhibitor</t>
+          <t>oral SERD</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
@@ -4576,7 +4580,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4586,12 +4594,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -4606,17 +4614,17 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+          <t>povetacicept (ALPN-303)</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>APOL1 inhibitor</t>
+          <t>dual BAFF/APRIL inhibitor</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>IgA nephropathy</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4629,11 +4637,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr">
-        <is>
-          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
-        </is>
-      </c>
+      <c r="K73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4643,7 +4647,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2027-04-01</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4653,27 +4657,27 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Bayer</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>BAYRY</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Lynkuet (elinzanetant) sNDA</t>
+          <t>giredestrant + everolimus</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>NK-1/NK-3 receptor antagonist</t>
+          <t>oral SERD + mTOR inhibitor</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
@@ -4686,64 +4690,174 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
-        </is>
-      </c>
+      <c r="K74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F75" s="3" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G75" s="3" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I77" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J75" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K75" s="3" t="inlineStr">
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
@@ -4826,6 +4940,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: split inaxaplin Phase 2b/Phase 3 catalysts and add Tukysa approval row (#282)
Co-authored-by: mps5cy@virginia.edu <mps5cy@virginia.edu>
Co-authored-by: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K75"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2915,42 +2915,42 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>VRTX</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Galleri MCED test</t>
+          <t>inaxaplin (AMPLIFIED Phase 2b)</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>multi-cancer early detection</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>cancer screening</t>
+          <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
+          <t>Phase 2b AMPLIFIED topline: UACR -42.7% in the modest-proteinuria cohort, -17.3% in the T2D cohort (CI crosses 0). Not the Phase 3 AMPLITUDE readout - see the 2026-09-30 and 2027-01-01 rows.</t>
         </is>
       </c>
     </row>
@@ -2977,42 +2977,42 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Mirum/Incyte</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>MIRM</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>Galleri MCED test</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>oral ALK2 kinase inhibitor</t>
+          <t>multi-cancer early detection</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+          <t>cancer screening</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
@@ -3022,19 +3022,19 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
+          <t>First-ever FDA AdComm on an MCED test (PMA) | Panel voted 10-0 safety, 6-4 effectiveness, 7-2-1 benefit-risk; supported use as adjunct, not substitute, for guideline screening. PMA decision pending, no date.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3044,27 +3044,27 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>superficial basal cell carcinoma (sBCC)</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3079,19 +3079,19 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3101,32 +3101,32 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I46" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
@@ -3136,14 +3136,14 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3158,32 +3158,32 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>hemophilia A</t>
+        </is>
+      </c>
+      <c r="I47" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3215,27 +3215,27 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Priovant/Roivant</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
+          <t>dermatomyositis</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
@@ -3272,27 +3272,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
+          <t>polycythemia vera</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3307,14 +3307,14 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3324,37 +3324,37 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>spinal muscular atrophy</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>positive</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | Resolved by Phase 2b AMPLIFIED (not AMPLITUDE): UACR -42.7% modest-proteinuria cohort, -17.3% T2D cohort (CI crosses 0). AMPLITUDE interim analysis tracked as separate row.</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
@@ -3376,38 +3376,42 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr"/>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>positive</t>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I51" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3417,54 +3421,50 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,54 +3474,54 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>Tukysa (tucatinib)</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>HER2-selective tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I53" s="7" t="inlineStr">
-        <is>
-          <t>withdrawn</t>
+          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,46 +3531,54 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
+          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr"/>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>CHMP monthly meeting</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr"/>
+          <t>Tecentriq (atezolizumab)</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>PD-L1 checkpoint inhibitor</t>
+        </is>
+      </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I54" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
@@ -3580,19 +3588,19 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3602,32 +3610,32 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Merck/Daiichi Sankyo</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>IL-6 receptor antagonist</t>
+          <t>B7-H3 antibody-drug conjugate</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>extensive-stage small cell lung cancer</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3637,49 +3645,41 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>VTRS</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -3716,32 +3716,32 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Enspryng (satralizumab)</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>IL-6 receptor antagonist</t>
         </is>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
-        </is>
-      </c>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3751,45 +3751,49 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>First IL-6R challenger to Tepezza</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>guidance</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr"/>
+          <t>Viatris/Opus Genetics</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>BsUFA IV reauthorization public meeting</t>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>biosimilars</t>
+          <t>alpha-adrenergic antagonist eye drop</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>presbyopia</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3804,7 +3808,7 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3820,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3826,32 +3830,32 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Pharming</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>PHAR</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>leniolisib</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>PI3K-delta inhibitor</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
-        </is>
-      </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3861,49 +3865,45 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>INO</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3918,49 +3918,49 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3975,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3997,27 +3997,27 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Agios</t>
+          <t>Inovio</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>INO</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>mitapivat (PYRUKYND)</t>
+          <t>INO-3107</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>pyruvate kinase activator</t>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>sickle cell disease (RISE UP)</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -4030,47 +4030,51 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K62" s="3" t="inlineStr"/>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Cytokinetics</t>
+          <t>Vaxcyte</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>CYTK</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>aficamten (MAPLE-HCM)</t>
+          <t>VAX-31</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>cardiac myosin inhibitor</t>
+          <t>31-valent pneumococcal conjugate vaccine</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>obstructive HCM (MAPLE-HCM label update)</t>
+          <t>adult pneumococcal disease prevention</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -4083,7 +4087,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K63" s="3" t="inlineStr"/>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4093,7 +4101,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4103,27 +4111,27 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Summit</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>ivonescimab</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>PD-1 x VEGF bispecific antibody</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>EGFR-mutant NSCLC with platinum doublet</t>
+          <t>sickle cell disease (RISE UP)</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -4136,43 +4144,47 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t>First US filing for the PD-1/VEGF bispecific class.</t>
-        </is>
-      </c>
+      <c r="K64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr"/>
+          <t>Cytokinetics</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>CYTK</t>
+        </is>
+      </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G65" s="3" t="inlineStr"/>
+          <t>aficamten (MAPLE-HCM)</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>cardiac myosin inhibitor</t>
+        </is>
+      </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -4185,21 +4197,17 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr">
-        <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
-        </is>
-      </c>
+      <c r="K65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4209,32 +4217,32 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
+          <t>Summit</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>CAPR</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>ivonescimab</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>PD-1 x VEGF bispecific antibody</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I66" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
+        </is>
+      </c>
+      <c r="I66" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr">
@@ -4244,49 +4252,41 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Savara</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>SVRA</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>MOLBREEVI (molgramostim)</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr">
-        <is>
-          <t>inhaled GM-CSF</t>
-        </is>
-      </c>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>autoimmune pulmonary alveolar proteinosis</t>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4301,19 +4301,19 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -4323,32 +4323,32 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>BridgeBio</t>
+          <t>Capricor</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>CAPR</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>BBP-418 (ribitol)</t>
+          <t>deramiocel</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>glycosylation substrate</t>
+          <t>allogeneic cell therapy</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
-        </is>
-      </c>
-      <c r="I68" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4356,7 +4356,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K68" s="3" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4366,7 +4370,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -4376,27 +4380,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Cogent</t>
+          <t>Savara</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>bezuclastinib + sunitinib</t>
+          <t>MOLBREEVI (molgramostim)</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>KIT inhibitor</t>
+          <t>inhaled GM-CSF</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>gastrointestinal stromal tumor (PEAK)</t>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -4411,7 +4415,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4427,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4433,27 +4437,27 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>BridgeBio</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>BBIO</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>giredestrant (adjuvant)</t>
+          <t>BBP-418 (ribitol)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>oral SERD</t>
+          <t>glycosylation substrate</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4466,11 +4470,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr">
-        <is>
-          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
-        </is>
-      </c>
+      <c r="K70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4490,27 +4490,27 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Cogent</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>COGT</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>povetacicept (ALPN-303)</t>
+          <t>bezuclastinib + sunitinib</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>dual BAFF/APRIL inhibitor</t>
+          <t>KIT inhibitor</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>IgA nephropathy</t>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4523,7 +4523,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4533,7 +4537,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4553,17 +4557,17 @@
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>giredestrant + everolimus</t>
+          <t>giredestrant (adjuvant)</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>oral SERD + mTOR inhibitor</t>
+          <t>oral SERD</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
@@ -4576,7 +4580,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4586,12 +4594,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -4606,17 +4614,17 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+          <t>povetacicept (ALPN-303)</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>APOL1 inhibitor</t>
+          <t>dual BAFF/APRIL inhibitor</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
+          <t>IgA nephropathy</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4629,11 +4637,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr">
-        <is>
-          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
-        </is>
-      </c>
+      <c r="K73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4643,7 +4647,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2027-04-01</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4653,27 +4657,27 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Bayer</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>BAYRY</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>Lynkuet (elinzanetant) sNDA</t>
+          <t>giredestrant + everolimus</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>NK-1/NK-3 receptor antagonist</t>
+          <t>oral SERD + mTOR inhibitor</t>
         </is>
       </c>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
@@ -4686,64 +4690,174 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
-        </is>
-      </c>
+      <c r="K74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F75" s="3" t="inlineStr">
+      <c r="F77" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G75" s="3" t="inlineStr">
+      <c r="G77" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I75" s="6" t="inlineStr">
+      <c r="I77" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J75" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K75" s="3" t="inlineStr">
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
@@ -4826,6 +4940,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: weekly brief + watchlist 2026-10-16
Resolves CHMP Oct, Enspryng TED (approved 10/15), VAX-31 OPUS-1 (positive 10/5).
Adds 9 rows (76 -> 85): BNT113 miss, CHMP opinions (Foundayo, Rasonque, Tukysa),
Anktiva papillary early approval, TumorSight Risk 510(k), SYD-101 AdComm 10/30,
CHMP Nov 9-12, Enspryng MOGAD PDUFA 1/10/27. Regenerates catalysts.xlsx.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Draft guidance on device presentations for biosimilars; comments due Oct 2 2026</t>
+          <t>Draft guidance on device presentations for biosimilars; comments due Oct 2 2026 | Oct 16: draft posted Jul 30 2026 (listed as a July 2026 Biosimilars Action Plan deliverable); comment period closed Oct 2. Left 'upcoming' because the status vocabulary has no 'published' value - schema decision pending.</t>
         </is>
       </c>
     </row>
@@ -3029,42 +3029,38 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Mirum/Incyte</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>MIRM</t>
-        </is>
-      </c>
+          <t>SimBioSys</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>TumorSight Risk (510(k))</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>oral ALK2 kinase inhibitor</t>
+          <t>AI MRI-derived prognostic software</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+          <t>5- and 10-year recurrence risk, HR+/HER2- stage I-IIIA breast cancer</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3079,19 +3075,19 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
+          <t>510(k) clearance decision dated Sep 25, announced Oct 15; predicate ArteraAI Breast. Retrospective validation n=2,129 (high vs low risk HR 3.3); no evidence yet that use changes treatment or outcomes. 'approved' = cleared.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3101,27 +3097,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>superficial basal cell carcinoma (sBCC)</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -3136,19 +3132,19 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3158,32 +3154,32 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3193,14 +3189,14 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3215,32 +3211,32 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>hemophilia A</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3250,7 +3246,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3272,27 +3268,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Priovant/Roivant</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
+          <t>dermatomyositis</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3307,7 +3303,7 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
@@ -3329,27 +3325,27 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
+          <t>polycythemia vera</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -3364,14 +3360,14 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3381,37 +3377,37 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
-        </is>
-      </c>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>spinal muscular atrophy</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3421,7 +3417,7 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
@@ -3433,38 +3429,42 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>positive</t>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,54 +3474,50 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Pfizer</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>PFE</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Tukysa (tucatinib)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>HER2-selective tyrosine kinase inhibitor</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,49 +3527,49 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>Tukysa (tucatinib)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>HER2-selective tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
+          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -3588,7 +3584,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
+          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3596,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3610,32 +3606,32 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>PD-L1 checkpoint inhibitor</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>withdrawn</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3645,46 +3641,54 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
+          <t>Merck/Daiichi Sankyo</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>CHMP monthly meeting</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr"/>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>B7-H3 antibody-drug conjugate</t>
+        </is>
+      </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>extensive-stage small cell lung cancer</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
@@ -3694,54 +3698,46 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>IL-6 receptor antagonist</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
-        </is>
-      </c>
-      <c r="I57" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3751,54 +3747,54 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13. | Oct 12-15 highlights: 6 new medicines positive (incl. Foundayo/orforglipron, Rasonque/daraxonrasib, Yuviwel, 2 biosimilars), 5 extensions (incl. Tukysa, Talvey, Tryngolza), Yartemlea refusal confirmed on re-examination.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
+          <t>BioNTech</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>VTRS</t>
+          <t>BNTX</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+          <t>BNT113 (AHEAD-MERIT)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
+          <t>mRNA cancer immunotherapy (HPV16 E6/E7)</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
-        </is>
-      </c>
-      <c r="I58" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>1L HPV16+ PD-L1 CPS&gt;=1 recurrent/metastatic HNSCC with pembrolizumab</t>
+        </is>
+      </c>
+      <c r="I58" s="8" t="inlineStr">
+        <is>
+          <t>negative</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -3808,54 +3804,54 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Missed first dual primary endpoint (PFS) vs pembrolizumab alone; no HR disclosed. IDMC: continue to OS, which could still make the trial positive. Shares -7%.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Eli Lilly</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Foundayo (orforglipron)</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>oral small-molecule GLP-1 receptor agonist</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
+          <t>obesity/weight management and type 2 diabetes in adults</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3865,50 +3861,54 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>Positive CHMP opinion for once-daily oral GLP-1 tablet; EC decision typically ~67 days later.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>guidance</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
+          <t>Pfizer</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>BsUFA IV reauthorization public meeting</t>
+          <t>Tukysa (tucatinib) extension</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>biosimilars</t>
+          <t>HER2 tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>maintenance with trastuzumab + pertuzumab in HER2+ unresectable/metastatic breast cancer after 1L induction</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
@@ -3918,54 +3918,54 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+          <t>EU extension follows US approval Oct 7 2026 (HER2CLIMB-05).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Revolution Medicines</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>Rasonque (daraxonrasib)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>oral RAS(ON) inhibitor</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
-        </is>
-      </c>
-      <c r="I61" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>metastatic pancreatic adenocarcinoma after &gt;=1 prior therapy</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
@@ -3975,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Phased review under EMA Cancer Medicines Pathfinder; RASolute 302. US approval Aug 26 2026.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3997,32 +3997,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>Enspryng (satralizumab)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>IL-6 receptor antagonist</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
-        </is>
-      </c>
-      <c r="I62" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -4032,49 +4032,49 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>First IL-6R challenger to Tepezza | Approved Oct 15 2026; first at-home SC TED therapy and first IL-6R inhibitor in TED. SatraGO-1 missed its week-24 primary endpoint; SatraGO-2 proptosis response 52.9% vs 23.4%. MOGAD sBLA PDUFA Jan 10 2027 tracked separately.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>Viatris/Opus Genetics</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>VTRS</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>alpha-adrenergic antagonist eye drop</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>presbyopia</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -4089,19 +4089,19 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4111,32 +4111,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Agios</t>
+          <t>Pharming</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>PHAR</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>mitapivat (PYRUKYND)</t>
+          <t>leniolisib</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>pyruvate kinase activator</t>
+          <t>PI3K-delta inhibitor</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>sickle cell disease (RISE UP)</t>
-        </is>
-      </c>
-      <c r="I64" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
@@ -4144,7 +4144,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4154,37 +4158,33 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Cytokinetics</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>CYTK</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>aficamten (MAPLE-HCM)</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>cardiac myosin inhibitor</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>obstructive HCM (MAPLE-HCM label update)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -4197,17 +4197,21 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4217,27 +4221,27 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Summit</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>ivonescimab</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>PD-1 x VEGF bispecific antibody</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>EGFR-mutant NSCLC with platinum doublet</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
@@ -4252,41 +4256,49 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr"/>
+          <t>Inovio</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr"/>
+          <t>INO-3107</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+        </is>
+      </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4301,54 +4313,50 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>CAPR</t>
-        </is>
-      </c>
+          <t>Sydnexis</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>SYD-101 (atropine sulfate ophthalmic solution 0.01%)</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>low-dose muscarinic antagonist</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I68" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>slowing myopia progression in children 3 years and older</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4358,54 +4366,54 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+          <t>Dermatologic and Ophthalmic Drugs AdComm on NDA 219694, which received a CRL in 2025. Docket FDA-2026-N-10606 closes Oct 29.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Savara</t>
+          <t>Vaxcyte</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>SVRA</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>MOLBREEVI (molgramostim)</t>
+          <t>VAX-31</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>inhaled GM-CSF</t>
+          <t>31-valent pneumococcal conjugate vaccine</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>autoimmune pulmonary alveolar proteinosis</t>
-        </is>
-      </c>
-      <c r="I69" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>adult pneumococcal disease prevention</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
@@ -4415,7 +4423,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31. | OPUS-1 (n=4,047) met all prespecified primary immunogenicity endpoints vs PCV20/PCV21; serotypes 3 and 12F missed the &gt;0.667 NI bar vs PCV21 in separate comparator analysis. OPUS-2/3 H1 2027; BLA planned H1 2028.</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4435,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4437,27 +4445,27 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>BridgeBio</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>BBP-418 (ribitol)</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>glycosylation substrate</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+          <t>sickle cell disease (RISE UP)</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4475,42 +4483,42 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Cogent</t>
+          <t>EMA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>bezuclastinib + sunitinib</t>
+          <t>CHMP monthly meeting</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>KIT inhibitor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>gastrointestinal stromal tumor (PEAK)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4525,7 +4533,7 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+          <t>Nov 9-12 2026 meeting; opinions typically published on the Friday after.</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4545,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4547,27 +4555,27 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Cytokinetics</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>CYTK</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>giredestrant (adjuvant)</t>
+          <t>aficamten (MAPLE-HCM)</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>oral SERD</t>
+          <t>cardiac myosin inhibitor</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
@@ -4580,11 +4588,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr">
-        <is>
-          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
-        </is>
-      </c>
+      <c r="K72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4594,7 +4598,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -4604,27 +4608,27 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Summit</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>povetacicept (ALPN-303)</t>
+          <t>ivonescimab</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>dual BAFF/APRIL inhibitor</t>
+          <t>PD-1 x VEGF bispecific antibody</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>IgA nephropathy</t>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4637,47 +4641,43 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>giredestrant + everolimus</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>oral SERD + mTOR inhibitor</t>
-        </is>
-      </c>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
@@ -4690,52 +4690,56 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Capricor</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>CAPR</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+          <t>deramiocel</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>APOL1 inhibitor</t>
+          <t>allogeneic cell therapy</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
-        </is>
-      </c>
-      <c r="I75" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
@@ -4745,7 +4749,7 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4761,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2027-04-01</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4767,27 +4771,27 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Bayer</t>
+          <t>Savara</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>BAYRY</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Lynkuet (elinzanetant) sNDA</t>
+          <t>MOLBREEVI (molgramostim)</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>NK-1/NK-3 receptor antagonist</t>
+          <t>inhaled GM-CSF</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4802,69 +4806,570 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>BridgeBio</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>BBIO</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>BBP-418 (ribitol)</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>glycosylation substrate</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Cogent</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>COGT</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>bezuclastinib + sunitinib</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>KIT inhibitor</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant (adjuvant)</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>povetacicept (ALPN-303)</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>dual BAFF/APRIL inhibitor</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant + everolimus</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD + mTOR inhibitor</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-06</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>ImmunityBio</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Anktiva (nogapendekin alfa inbakicept) + BCG</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>IL-15 superagonist</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>BCG-unresponsive high-grade papillary-only NMIBC</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>Approved ~12 weeks early by extrapolating CIS efficacy (n=77, CR 62%) to papillary-only disease; FDA refused to file this application in May 2025. FDA calls it 'a new FDA approach'. Jan 6 2027 action date per BioMed Nexus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-10</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Enspryng (satralizumab) MOGAD sBLA</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>IL-6 receptor antibody</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>myelin oligodendrocyte glycoprotein antibody-associated disease (METEOROID)</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>Priority review; no approved MOGAD therapies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F77" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr">
+      <c r="I86" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J77" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K77" s="3" t="inlineStr">
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K75"/>
+  <autoFilter ref="A1:K86"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -4942,6 +5447,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
intel: weekly brief + watchlist 2026-10-16 (#283)
Resolves CHMP Oct, Enspryng TED (approved 10/15), VAX-31 OPUS-1 (positive 10/5).
Adds 9 rows (76 -> 85): BNT113 miss, CHMP opinions (Foundayo, Rasonque, Tukysa),
Anktiva papillary early approval, TumorSight Risk 510(k), SYD-101 AdComm 10/30,
CHMP Nov 9-12, Enspryng MOGAD PDUFA 1/10/27. Regenerates catalysts.xlsx.

Co-authored-by: maekass <234696301+maekass@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Draft guidance on device presentations for biosimilars; comments due Oct 2 2026</t>
+          <t>Draft guidance on device presentations for biosimilars; comments due Oct 2 2026 | Oct 16: draft posted Jul 30 2026 (listed as a July 2026 Biosimilars Action Plan deliverable); comment period closed Oct 2. Left 'upcoming' because the status vocabulary has no 'published' value - schema decision pending.</t>
         </is>
       </c>
     </row>
@@ -3029,42 +3029,38 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Mirum/Incyte</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>MIRM</t>
-        </is>
-      </c>
+          <t>SimBioSys</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>zilurgisertib</t>
+          <t>TumorSight Risk (510(k))</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>oral ALK2 kinase inhibitor</t>
+          <t>AI MRI-derived prognostic software</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
+          <t>5- and 10-year recurrence risk, HR+/HER2- stage I-IIIA breast cancer</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -3079,19 +3075,19 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
+          <t>510(k) clearance decision dated Sep 25, announced Oct 15; predicate ArteraAI Breast. Retrospective validation n=2,129 (high vs low risk HR 3.3); no evidence yet that use changes treatment or outcomes. 'approved' = cleared.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3101,27 +3097,27 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Mirum/Incyte</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
+          <t>MIRM</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>Ameluz + RhodoLED lamp series</t>
+          <t>zilurgisertib</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>photodynamic therapy</t>
+          <t>oral ALK2 kinase inhibitor</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>superficial basal cell carcinoma (sBCC)</t>
+          <t>fibrodysplasia ossificans progressiva (FOP), patients 12 and older</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -3136,19 +3132,19 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
+          <t>CORRECTED 2026-09-18: this row previously read 'anemia of myelofibrosis' on the strength of a pdufa.bio listing. The NDA is for FOP, accepted under Priority Review with a Sep 26 2026 goal date; Mirum licensed worldwide rights from Incyte in May 2026. Third aggregator error caught in this file - do not seed indications from calendar sites. | Approved Sep 25 2026 as Atebrioz for FOP age 12+; rare pediatric PRV issued to Incyte.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3158,32 +3154,32 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>BFRI</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Mim8 (denecimig)</t>
+          <t>Ameluz + RhodoLED lamp series</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>FVIII-mimetic bispecific antibody</t>
+          <t>photodynamic therapy</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I47" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>superficial basal cell carcinoma (sBCC)</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
@@ -3193,14 +3189,14 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
+          <t>Device-drug combination label expansion | Approved Sep 14 2026, two weeks before PDUFA; indication is superficial basal cell carcinoma (sBCC), not AK - prior indication field was the existing label.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3215,32 +3211,32 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>brepocitinib</t>
+          <t>Mim8 (denecimig)</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>TYK2/JAK1 inhibitor</t>
+          <t>FVIII-mimetic bispecific antibody</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>approved</t>
+          <t>hemophilia A</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
@@ -3250,7 +3246,7 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>Next-gen challenger to Hemlibra | Oct 2 2026: FDA review extended over facility remediation after pre-license inspection; no clinical deficiencies cited; no new action date; Novo targets US launch H1 2027. CHMP positive Sep 17 (Frehemgo).</t>
         </is>
       </c>
     </row>
@@ -3272,27 +3268,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>Priovant/Roivant</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
+          <t>ROIV</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>rusfertide</t>
+          <t>brepocitinib</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>hepcidin mimetic</t>
+          <t>TYK2/JAK1 inhibitor</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>polycythemia vera</t>
+          <t>dermatomyositis</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -3307,7 +3303,7 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
@@ -3329,27 +3325,27 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>PTGX</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>apitegromab</t>
+          <t>rusfertide</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>anti-myostatin antibody</t>
+          <t>hepcidin mimetic</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>spinal muscular atrophy</t>
+          <t>polycythemia vera</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -3364,14 +3360,14 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3381,37 +3377,37 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SRRK</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (VX-147)</t>
+          <t>apitegromab</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>APOL1 channel function inhibitor</t>
+          <t>anti-myostatin antibody</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
-        </is>
-      </c>
-      <c r="I51" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>spinal muscular atrophy</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -3421,7 +3417,7 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
@@ -3433,38 +3429,42 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr"/>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>Vaccines and Related Biological Products Advisory Committee</t>
+          <t>inaxaplin (VX-147)</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>influenza vaccines</t>
+          <t>APOL1 channel function inhibitor</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>positive</t>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I52" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
@@ -3474,54 +3474,50 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window | No Phase 3 AMPLITUDE data in the Sep 30 window: Vertex now guides the AMPLITUDE interim analysis for early 2027 (tracked as the 2027-01-01 row). The Sep 22 result was Phase 2b AMPLIFIED, tracked as its own row.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Pfizer</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>PFE</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Tukysa (tucatinib)</t>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>HER2-selective tyrosine kinase inhibitor</t>
+          <t>influenza vaccines</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -3531,49 +3527,49 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session | Committee voted 9-0 for WHO-matched trivalent 2027 SH egg-based composition.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Pfizer</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>PFE</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>Tukysa (tucatinib)</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>PD-L1 checkpoint inhibitor</t>
+          <t>HER2-selective tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>stage III colon cancer</t>
+          <t>HER2+ metastatic breast cancer, first-line maintenance with trastuzumab and pertuzumab (HER2CLIMB-05)</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -3588,7 +3584,7 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
+          <t>Approved Oct 7 2026 with trastuzumab and pertuzumab as maintenance therapy for HER2+ metastatic breast cancer. HER2CLIMB-05 median PFS 24.9 vs 16.3 months (HR 0.64). Label carries a boxed hepatotoxicity warning per Drugs.com.</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3596,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -3610,32 +3606,32 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>B7-H3 antibody-drug conjugate</t>
+          <t>PD-L1 checkpoint inhibitor</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>withdrawn</t>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -3645,46 +3641,54 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
+          <t>Checkpoint expansion into adjuvant colon | Approved Oct 8 2026 (IV and SC Hybreza) with FOLFOX for adjuvant stage III dMMR colon cancer; ATOMIC DFS HR 0.50. 12th US indication.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr"/>
+          <t>Merck/Daiichi Sankyo</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>CHMP monthly meeting</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr"/>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>B7-H3 antibody-drug conjugate</t>
+        </is>
+      </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I56" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>extensive-stage small cell lung cancer</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
@@ -3694,54 +3698,46 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13.</t>
+          <t>First regulatory decision for a B7-H3 ADC | BLA voluntarily withdrawn Sep 25 2026 after FDA said single-arm Phase 2 IDeate-Lung01 data did not support accelerated approval; path now via Phase 3 IDeate-Lung02.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr"/>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>Enspryng (satralizumab)</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>IL-6 receptor antagonist</t>
-        </is>
-      </c>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr"/>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>thyroid eye disease</t>
-        </is>
-      </c>
-      <c r="I57" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -3751,54 +3747,54 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>Oct 12-15 plenary per EMA's published 2026 meeting-dates document. Watch the EC decisions on this month's ovarian-cancer and biosimilar opinions. | Meeting runs Oct 12-15 2026; opinions not yet published as of Oct 13. | Oct 12-15 highlights: 6 new medicines positive (incl. Foundayo/orforglipron, Rasonque/daraxonrasib, Yuviwel, 2 biosimilars), 5 extensions (incl. Tukysa, Talvey, Tryngolza), Yartemlea refusal confirmed on re-examination.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Viatris/Opus Genetics</t>
+          <t>BioNTech</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>VTRS</t>
+          <t>BNTX</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+          <t>BNT113 (AHEAD-MERIT)</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>alpha-adrenergic antagonist eye drop</t>
+          <t>mRNA cancer immunotherapy (HPV16 E6/E7)</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>presbyopia</t>
-        </is>
-      </c>
-      <c r="I58" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>1L HPV16+ PD-L1 CPS&gt;=1 recurrent/metastatic HNSCC with pembrolizumab</t>
+        </is>
+      </c>
+      <c r="I58" s="8" t="inlineStr">
+        <is>
+          <t>negative</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -3808,54 +3804,54 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+          <t>Missed first dual primary endpoint (PFS) vs pembrolizumab alone; no HR disclosed. IDMC: continue to OS, which could still make the trial positive. Shares -7%.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Eli Lilly</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>leniolisib</t>
+          <t>Foundayo (orforglipron)</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>PI3K-delta inhibitor</t>
+          <t>oral small-molecule GLP-1 receptor agonist</t>
         </is>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
+          <t>obesity/weight management and type 2 diabetes in adults</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>positive</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
@@ -3865,50 +3861,54 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+          <t>Positive CHMP opinion for once-daily oral GLP-1 tablet; EC decision typically ~67 days later.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>guidance</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr"/>
+          <t>Pfizer</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>PFE</t>
+        </is>
+      </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>BsUFA IV reauthorization public meeting</t>
+          <t>Tukysa (tucatinib) extension</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>biosimilars</t>
+          <t>HER2 tyrosine kinase inhibitor</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I60" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>maintenance with trastuzumab + pertuzumab in HER2+ unresectable/metastatic breast cancer after 1L induction</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
@@ -3918,54 +3918,54 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+          <t>EU extension follows US approval Oct 7 2026 (HER2CLIMB-05).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Revolution Medicines</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>RVMD</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>bepirovirsen</t>
+          <t>Rasonque (daraxonrasib)</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>antisense oligonucleotide</t>
+          <t>oral RAS(ON) inhibitor</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>chronic hepatitis B</t>
-        </is>
-      </c>
-      <c r="I61" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>metastatic pancreatic adenocarcinoma after &gt;=1 prior therapy</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
@@ -3975,19 +3975,19 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+          <t>Phased review under EMA Cancer Medicines Pathfinder; RASolute 302. US approval Aug 26 2026.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -3997,32 +3997,32 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Inovio</t>
+          <t>Roche</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>INO</t>
+          <t>RHHBY</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>INO-3107</t>
+          <t>Enspryng (satralizumab)</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+          <t>IL-6 receptor antagonist</t>
         </is>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>recurrent respiratory papillomatosis</t>
-        </is>
-      </c>
-      <c r="I62" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
@@ -4032,49 +4032,49 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+          <t>First IL-6R challenger to Tepezza | Approved Oct 15 2026; first at-home SC TED therapy and first IL-6R inhibitor in TED. SatraGO-1 missed its week-24 primary endpoint; SatraGO-2 proptosis response 52.9% vs 23.4%. MOGAD sBLA PDUFA Jan 10 2027 tracked separately.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Vaxcyte</t>
+          <t>Viatris/Opus Genetics</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>PCVX</t>
+          <t>VTRS</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>VAX-31</t>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>31-valent pneumococcal conjugate vaccine</t>
+          <t>alpha-adrenergic antagonist eye drop</t>
         </is>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>adult pneumococcal disease prevention</t>
+          <t>presbyopia</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -4089,19 +4089,19 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31.</t>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2026-11-01</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4111,32 +4111,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Agios</t>
+          <t>Pharming</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>PHAR</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>mitapivat (PYRUKYND)</t>
+          <t>leniolisib</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>pyruvate kinase activator</t>
+          <t>PI3K-delta inhibitor</t>
         </is>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>sickle cell disease (RISE UP)</t>
-        </is>
-      </c>
-      <c r="I64" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
@@ -4144,7 +4144,11 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K64" s="3" t="inlineStr"/>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4154,37 +4158,33 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>guidance</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Cytokinetics</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>CYTK</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>aficamten (MAPLE-HCM)</t>
+          <t>BsUFA IV reauthorization public meeting</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>cardiac myosin inhibitor</t>
+          <t>biosimilars</t>
         </is>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
-          <t>obstructive HCM (MAPLE-HCM label update)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -4197,17 +4197,21 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Draft BsUFA IV commitment letter (Sep 24) proposes 4/6-month supplement reviews, provisional approval, late-review extension for resolvable issues. Docket closes Nov 25. Interchangeability strategy document comments due Nov 17.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -4217,27 +4221,27 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Summit</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>SMMT</t>
+          <t>GSK</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>ivonescimab</t>
+          <t>bepirovirsen</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>PD-1 x VEGF bispecific antibody</t>
+          <t>antisense oligonucleotide</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>EGFR-mutant NSCLC with platinum doublet</t>
+          <t>chronic hepatitis B</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
@@ -4252,41 +4256,49 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+          <t>B-Well program; functional-cure ambition in HBV</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr"/>
+          <t>Inovio</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Microbiology Devices Panel</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr"/>
+          <t>INO-3107</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+        </is>
+      </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
+          <t>recurrent respiratory papillomatosis</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4301,54 +4313,50 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Capricor</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>CAPR</t>
-        </is>
-      </c>
+          <t>Sydnexis</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>deramiocel</t>
+          <t>SYD-101 (atropine sulfate ophthalmic solution 0.01%)</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>allogeneic cell therapy</t>
+          <t>low-dose muscarinic antagonist</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>DMD cardiomyopathy</t>
-        </is>
-      </c>
-      <c r="I68" s="9" t="inlineStr">
-        <is>
-          <t>delayed</t>
+          <t>slowing myopia progression in children 3 years and older</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4358,54 +4366,54 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
+          <t>Dermatologic and Ophthalmic Drugs AdComm on NDA 219694, which received a CRL in 2025. Docket FDA-2026-N-10606 closes Oct 29.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Savara</t>
+          <t>Vaxcyte</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>SVRA</t>
+          <t>PCVX</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>MOLBREEVI (molgramostim)</t>
+          <t>VAX-31</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>inhaled GM-CSF</t>
+          <t>31-valent pneumococcal conjugate vaccine</t>
         </is>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>autoimmune pulmonary alveolar proteinosis</t>
-        </is>
-      </c>
-      <c r="I69" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>adult pneumococcal disease prevention</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
         </is>
       </c>
       <c r="J69" s="5" t="inlineStr">
@@ -4415,7 +4423,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
+          <t>OPUS-1 Phase 3 pivotal non-inferiority topline (safety, tolerability, immunogenicity) guided to the end of October 2026; month-precision placeholder at 2026-10-31. | OPUS-1 (n=4,047) met all prespecified primary immunogenicity endpoints vs PCV20/PCV21; serotypes 3 and 12F missed the &gt;0.667 NI bar vs PCV21 in separate comparator analysis. OPUS-2/3 H1 2027; BLA planned H1 2028.</t>
         </is>
       </c>
     </row>
@@ -4427,7 +4435,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-11-01</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4437,27 +4445,27 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>BridgeBio</t>
+          <t>Agios</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>BBIO</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>BBP-418 (ribitol)</t>
+          <t>mitapivat (PYRUKYND)</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>glycosylation substrate</t>
+          <t>pyruvate kinase activator</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+          <t>sickle cell disease (RISE UP)</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4475,42 +4483,42 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Cogent</t>
+          <t>EMA</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>COGT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>bezuclastinib + sunitinib</t>
+          <t>CHMP monthly meeting</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>KIT inhibitor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>gastrointestinal stromal tumor (PEAK)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4525,7 +4533,7 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+          <t>Nov 9-12 2026 meeting; opinions typically published on the Friday after.</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4545,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -4547,27 +4555,27 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Cytokinetics</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
+          <t>CYTK</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>giredestrant (adjuvant)</t>
+          <t>aficamten (MAPLE-HCM)</t>
         </is>
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>oral SERD</t>
+          <t>cardiac myosin inhibitor</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+          <t>obstructive HCM (MAPLE-HCM label update)</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
@@ -4580,11 +4588,7 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr">
-        <is>
-          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
-        </is>
-      </c>
+      <c r="K72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4594,7 +4598,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -4604,27 +4608,27 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Summit</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>SMMT</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>povetacicept (ALPN-303)</t>
+          <t>ivonescimab</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>dual BAFF/APRIL inhibitor</t>
+          <t>PD-1 x VEGF bispecific antibody</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>IgA nephropathy</t>
+          <t>EGFR-mutant NSCLC with platinum doublet</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4637,47 +4641,43 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>First US filing for the PD-1/VEGF bispecific class.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>2026-12-18</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>giredestrant + everolimus</t>
-        </is>
-      </c>
-      <c r="G74" s="3" t="inlineStr">
-        <is>
-          <t>oral SERD + mTOR inhibitor</t>
-        </is>
-      </c>
+          <t>Microbiology Devices Panel</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
       <c r="H74" s="3" t="inlineStr">
         <is>
-          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+          <t>pathogen-agnostic sequencing for outbreak preparedness and response</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
@@ -4690,52 +4690,56 @@
           <t>source</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Newly announced Sep 14 2026. Panel will advise on design, development and bioinformatics validation of pathogen-agnostic sequencing tests for known and unknown pathogens. No named sponsor or device - a framework session, relevant to sequencing diagnostics regulatory precedent. 9:00 a.m.-4:00 p.m. ET, White Oak.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>2027-01-01</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>PDUFA</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Vertex</t>
+          <t>Capricor</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>VRTX</t>
+          <t>CAPR</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+          <t>deramiocel</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>APOL1 inhibitor</t>
+          <t>allogeneic cell therapy</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>APOL1-mediated kidney disease</t>
-        </is>
-      </c>
-      <c r="I75" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
+          <t>DMD cardiomyopathy</t>
+        </is>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>delayed</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
@@ -4745,7 +4749,7 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+          <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4761,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>2027-04-01</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4767,27 +4771,27 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Bayer</t>
+          <t>Savara</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>BAYRY</t>
+          <t>SVRA</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>Lynkuet (elinzanetant) sNDA</t>
+          <t>MOLBREEVI (molgramostim)</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>NK-1/NK-3 receptor antagonist</t>
+          <t>inhaled GM-CSF</t>
         </is>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+          <t>autoimmune pulmonary alveolar proteinosis</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4802,69 +4806,570 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+          <t>Extended from Aug 22 after major amendment; sponsor says no safety/efficacy/CMC concerns cited.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>BridgeBio</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>BBIO</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>BBP-418 (ribitol)</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>glycosylation substrate</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>limb-girdle muscular dystrophy 2I/R9 (FORTIFY)</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Cogent</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>COGT</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>bezuclastinib + sunitinib</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>KIT inhibitor</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>gastrointestinal stromal tumor (PEAK)</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Second Cogent PDUFA (non-advanced systemic mastocytosis) Dec 30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant (adjuvant)</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>ER+/HER2- stage I-III early breast cancer (lidERA)</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>Priority review. lidERA iDFS HR 0.70 vs SOC endocrine therapy. Would be first oral SERD in the adjuvant setting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>povetacicept (ALPN-303)</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>dual BAFF/APRIL inhibitor</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>IgA nephropathy</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>giredestrant + everolimus</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD + mTOR inhibitor</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>ESR1-mutated ER+/HER2- advanced breast cancer (evERA)</t>
+        </is>
+      </c>
+      <c r="I81" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>readout</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Vertex</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (AMPLITUDE interim analysis)</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>Company guides 'early 2027'; quarter-precision placeholder. Positive IA could support US accelerated approval on one-year eGFR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-06</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>ImmunityBio</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>IBRX</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Anktiva (nogapendekin alfa inbakicept) + BCG</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>IL-15 superagonist</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>BCG-unresponsive high-grade papillary-only NMIBC</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>Approved ~12 weeks early by extrapolating CIS efficacy (n=77, CR 62%) to papillary-only disease; FDA refused to file this application in May 2025. FDA calls it 'a new FDA approach'. Jan 6 2027 action date per BioMed Nexus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>2027-01-10</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Enspryng (satralizumab) MOGAD sBLA</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>IL-6 receptor antibody</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>myelin oligodendrocyte glycoprotein antibody-associated disease (METEOROID)</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>Priority review; no approved MOGAD therapies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>2027-04-01</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Bayer</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Lynkuet (elinzanetant) sNDA</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>NK-1/NK-3 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>vasomotor symptoms from endocrine therapy for HR+ breast cancer (OASIS-4)</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>sNDA accepted with Priority Review Sep 28 2026; Bayer did not disclose the action date. Quarter placeholder is an ESTIMATE, not a sponsor date. Would be first US-approved therapy for ET-induced VMS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>2027-04-01</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Organon/Sebela Women's Health</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>OGN</t>
         </is>
       </c>
-      <c r="F77" s="3" t="inlineStr">
+      <c r="F86" s="3" t="inlineStr">
         <is>
           <t>MIUDELLA (copper intrauterine system)</t>
         </is>
       </c>
-      <c r="G77" s="3" t="inlineStr">
+      <c r="G86" s="3" t="inlineStr">
         <is>
           <t>hormone-free copper intrauterine device</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="H86" s="3" t="inlineStr">
         <is>
           <t>prevention of pregnancy - extension of duration of use to 6 years</t>
         </is>
       </c>
-      <c r="I77" s="6" t="inlineStr">
+      <c r="I86" s="6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J77" s="5" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="K77" s="3" t="inlineStr">
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
         <is>
           <t>sNDA accepted for review, announced Sep 14 2026; PDUFA action expected in Q2 calendar 2027, so scheduled_date is a quarter-precision placeholder at 2027-04-01. Current label is up to 3 years. Doubling labelled duration changes the per-patient economics of the only hormone-free IUD approved in the US.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K75"/>
+  <autoFilter ref="A1:K86"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -4942,6 +5447,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J76" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J86" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>